<commit_message>
updated final devoicing stimuli
</commit_message>
<xml_diff>
--- a/Dataset/stimuli_counting.xlsx
+++ b/Dataset/stimuli_counting.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ivy/Desktop/Modeling/SubInPhon/Seq2SeqModel/Dataset/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ivy/Desktop/Modeling/SubtanceInPhonology/Seq2SeqModel/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2366B78-379C-B74E-A348-A353982AD2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50518CC0-BC98-984C-9A1A-9914AD2B4518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="740" windowWidth="24960" windowHeight="15980" xr2:uid="{365D76DA-B6A5-5443-BBA8-94D6013D0945}"/>
+    <workbookView xWindow="-3780" yWindow="-17420" windowWidth="21760" windowHeight="15980" activeTab="1" xr2:uid="{365D76DA-B6A5-5443-BBA8-94D6013D0945}"/>
   </bookViews>
   <sheets>
-    <sheet name="English" sheetId="1" r:id="rId1"/>
-    <sheet name="Cantonese" sheetId="2" r:id="rId2"/>
+    <sheet name="EnglishBH" sheetId="1" r:id="rId1"/>
+    <sheet name="EnglishFD" sheetId="3" r:id="rId2"/>
+    <sheet name="CantoneseBH" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="47">
   <si>
     <t>V-CV</t>
   </si>
@@ -154,6 +155,30 @@
   </si>
   <si>
     <t>17 coda</t>
+  </si>
+  <si>
+    <t>14 onset</t>
+  </si>
+  <si>
+    <t>8 vowel</t>
+  </si>
+  <si>
+    <t>7 voiceless coda</t>
+  </si>
+  <si>
+    <t>7 voiced coda</t>
+  </si>
+  <si>
+    <t>VCVC</t>
+  </si>
+  <si>
+    <t>CVCVC</t>
+  </si>
+  <si>
+    <t>s4</t>
+  </si>
+  <si>
+    <t>s5</t>
   </si>
 </sst>
 </file>
@@ -623,17 +648,14 @@
         <v>578</v>
       </c>
       <c r="C4" s="2">
-        <f t="shared" ref="C4:E4" si="1">17*2*17</f>
+        <f t="shared" ref="C4:D4" si="1">17*2*17</f>
         <v>578</v>
       </c>
       <c r="D4" s="2">
         <f t="shared" si="1"/>
         <v>578</v>
       </c>
-      <c r="E4" s="2">
-        <f t="shared" si="1"/>
-        <v>578</v>
-      </c>
+      <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
@@ -649,7 +671,6 @@
       <c r="E5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="3"/>
       <c r="G5" s="1" t="s">
         <v>32</v>
       </c>
@@ -681,7 +702,6 @@
         <f>B6*C6*D6</f>
         <v>272</v>
       </c>
-      <c r="F6" s="3"/>
       <c r="G6" s="1">
         <v>4</v>
       </c>
@@ -712,10 +732,9 @@
         <v>1</v>
       </c>
       <c r="E7" s="1">
-        <f>B7*C7*D7+E6</f>
+        <f t="shared" ref="E7:E29" si="2">B7*C7*D7+E6</f>
         <v>4896</v>
       </c>
-      <c r="F7" s="3"/>
       <c r="G7" s="1">
         <v>4</v>
       </c>
@@ -747,10 +766,9 @@
         <v>1</v>
       </c>
       <c r="E8" s="1">
-        <f>B8*C8*D8+E7</f>
+        <f t="shared" si="2"/>
         <v>9520</v>
       </c>
-      <c r="F8" s="3"/>
       <c r="G8" s="1">
         <f>17*4</f>
         <v>68</v>
@@ -783,12 +801,11 @@
         <v>1</v>
       </c>
       <c r="E9" s="1">
-        <f>B9*C9*D9+E8</f>
+        <f t="shared" si="2"/>
         <v>88128</v>
       </c>
-      <c r="F9" s="3"/>
       <c r="G9" s="1">
-        <f t="shared" ref="G9:G11" si="2">17*4</f>
+        <f t="shared" ref="G9:G11" si="3">17*4</f>
         <v>68</v>
       </c>
       <c r="H9" s="1">
@@ -818,12 +835,11 @@
         <v>1</v>
       </c>
       <c r="E10" s="1">
-        <f>B10*C10*D10+E9</f>
+        <f t="shared" si="2"/>
         <v>88400</v>
       </c>
-      <c r="F10" s="3"/>
       <c r="G10" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>68</v>
       </c>
       <c r="H10" s="1">
@@ -853,12 +869,11 @@
         <v>1</v>
       </c>
       <c r="E11" s="1">
-        <f>B11*C11*D11+E10</f>
+        <f t="shared" si="2"/>
         <v>93024</v>
       </c>
-      <c r="F11" s="3"/>
       <c r="G11" s="1">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>68</v>
       </c>
       <c r="H11" s="1">
@@ -869,7 +884,7 @@
         <v>1</v>
       </c>
       <c r="J11" s="1">
-        <f t="shared" ref="J8:J13" si="3">G11*H11*I11+J10</f>
+        <f t="shared" ref="J11:J12" si="4">G11*H11*I11+J10</f>
         <v>88264</v>
       </c>
     </row>
@@ -888,10 +903,9 @@
         <v>1</v>
       </c>
       <c r="E12" s="1">
-        <f>B12*C12*D12+E11</f>
+        <f t="shared" si="2"/>
         <v>97648</v>
       </c>
-      <c r="F12" s="3"/>
       <c r="G12" s="1">
         <f>17*4*17</f>
         <v>1156</v>
@@ -903,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="J12" s="1">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>92888</v>
       </c>
     </row>
@@ -926,7 +940,6 @@
         <f>B13*C13*D13+E12</f>
         <v>176256</v>
       </c>
-      <c r="F13" s="3"/>
       <c r="G13" s="1">
         <f>17*4*17</f>
         <v>1156</v>
@@ -957,7 +970,7 @@
         <v>68</v>
       </c>
       <c r="E14">
-        <f>B14*C14*D14+E13</f>
+        <f t="shared" si="2"/>
         <v>194752</v>
       </c>
     </row>
@@ -975,7 +988,7 @@
         <v>1156</v>
       </c>
       <c r="E15">
-        <f>B15*C15*D15+E14</f>
+        <f t="shared" si="2"/>
         <v>509184</v>
       </c>
     </row>
@@ -993,7 +1006,7 @@
         <v>4</v>
       </c>
       <c r="E16">
-        <f>B16*C16*D16+E15</f>
+        <f t="shared" si="2"/>
         <v>527680</v>
       </c>
     </row>
@@ -1011,7 +1024,7 @@
         <v>68</v>
       </c>
       <c r="E17">
-        <f>B17*C17*D17+E16</f>
+        <f t="shared" si="2"/>
         <v>842112</v>
       </c>
     </row>
@@ -1029,7 +1042,7 @@
         <v>68</v>
       </c>
       <c r="E18">
-        <f>B18*C18*D18+E17</f>
+        <f t="shared" si="2"/>
         <v>1156544</v>
       </c>
     </row>
@@ -1047,7 +1060,7 @@
         <v>1156</v>
       </c>
       <c r="E19">
-        <f>B19*C19*D19+E18</f>
+        <f t="shared" si="2"/>
         <v>6501888</v>
       </c>
     </row>
@@ -1065,7 +1078,7 @@
         <v>4</v>
       </c>
       <c r="E20">
-        <f>B20*C20*D20+E19</f>
+        <f t="shared" si="2"/>
         <v>6816320</v>
       </c>
     </row>
@@ -1083,7 +1096,7 @@
         <v>68</v>
       </c>
       <c r="E21">
-        <f>B21*C21*D21+E20</f>
+        <f t="shared" si="2"/>
         <v>12161664</v>
       </c>
     </row>
@@ -1101,7 +1114,7 @@
         <v>68</v>
       </c>
       <c r="E22">
-        <f>B22*C22*D22+E21</f>
+        <f t="shared" si="2"/>
         <v>12180160</v>
       </c>
     </row>
@@ -1119,7 +1132,7 @@
         <v>1156</v>
       </c>
       <c r="E23">
-        <f>B23*C23*D23+E22</f>
+        <f t="shared" si="2"/>
         <v>12494592</v>
       </c>
     </row>
@@ -1137,7 +1150,7 @@
         <v>4</v>
       </c>
       <c r="E24">
-        <f>B24*C24*D24+E23</f>
+        <f t="shared" si="2"/>
         <v>12513088</v>
       </c>
     </row>
@@ -1155,7 +1168,7 @@
         <v>68</v>
       </c>
       <c r="E25">
-        <f>B25*C25*D25+E24</f>
+        <f t="shared" si="2"/>
         <v>12827520</v>
       </c>
     </row>
@@ -1173,7 +1186,7 @@
         <v>68</v>
       </c>
       <c r="E26">
-        <f>B26*C26*D26+E25</f>
+        <f t="shared" si="2"/>
         <v>13141952</v>
       </c>
     </row>
@@ -1191,7 +1204,7 @@
         <v>1156</v>
       </c>
       <c r="E27">
-        <f>B27*C27*D27+E26</f>
+        <f t="shared" si="2"/>
         <v>18487296</v>
       </c>
     </row>
@@ -1209,7 +1222,7 @@
         <v>4</v>
       </c>
       <c r="E28">
-        <f>B28*C28*D28+E27</f>
+        <f t="shared" si="2"/>
         <v>18801728</v>
       </c>
     </row>
@@ -1227,7 +1240,7 @@
         <v>68</v>
       </c>
       <c r="E29">
-        <f>B29*C29*D29+E28</f>
+        <f t="shared" si="2"/>
         <v>24147072</v>
       </c>
     </row>
@@ -1237,6 +1250,261 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEBC4378-3A0A-2749-A59B-9F52507C3F19}">
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>8</v>
+      </c>
+      <c r="F3" s="1">
+        <v>14</v>
+      </c>
+      <c r="G3" s="1">
+        <f>B3*C3*D3*E3*F3</f>
+        <v>112</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1</v>
+      </c>
+      <c r="D4" s="1">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1">
+        <v>8</v>
+      </c>
+      <c r="F4" s="1">
+        <v>14</v>
+      </c>
+      <c r="G4" s="1">
+        <f>B4*C4*D4*E4*F4+G3</f>
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="1">
+        <v>1</v>
+      </c>
+      <c r="C5" s="1">
+        <v>8</v>
+      </c>
+      <c r="D5" s="1">
+        <v>14</v>
+      </c>
+      <c r="E5" s="1">
+        <v>8</v>
+      </c>
+      <c r="F5" s="1">
+        <v>14</v>
+      </c>
+      <c r="G5" s="1">
+        <f>B5*C5*D5*E5*F5+G4</f>
+        <v>14224</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B6" s="1">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1">
+        <v>8</v>
+      </c>
+      <c r="D6" s="1">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1">
+        <v>8</v>
+      </c>
+      <c r="F6" s="1">
+        <v>14</v>
+      </c>
+      <c r="G6" s="1">
+        <f>B6*C6*D6*E6*F6+G5</f>
+        <v>189840</v>
+      </c>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="3"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="3"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5314F9FE-FDE3-3847-837A-D6395835C688}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
debugged input and return type
</commit_message>
<xml_diff>
--- a/Dataset/stimuli_counting.xlsx
+++ b/Dataset/stimuli_counting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ivy/Desktop/Modeling/SubtanceInPhonology/SubInPhon.nosync/Dataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C818209B-408B-5042-A08B-5BC1FE3444E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C792D7C4-E62B-E949-8037-3BCAB02A5291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4440" yWindow="740" windowWidth="24960" windowHeight="17920" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="52">
   <si>
     <t>V</t>
   </si>
@@ -115,48 +115,12 @@
     <t>V.CV-CVC</t>
   </si>
   <si>
-    <t>V.CVC-V</t>
-  </si>
-  <si>
-    <t>V.CVC-VC</t>
-  </si>
-  <si>
     <t>CV.CV-CV</t>
   </si>
   <si>
     <t>CV.CV-CVC</t>
   </si>
   <si>
-    <t>CV.CVC-V</t>
-  </si>
-  <si>
-    <t>CV.CVC-VC</t>
-  </si>
-  <si>
-    <t>VC.V-CV</t>
-  </si>
-  <si>
-    <t>VC.V-CVC</t>
-  </si>
-  <si>
-    <t>VC.VC-V</t>
-  </si>
-  <si>
-    <t>VC.VC-VC</t>
-  </si>
-  <si>
-    <t>CVC.V-CV</t>
-  </si>
-  <si>
-    <t>CVC.V-CVC</t>
-  </si>
-  <si>
-    <t>CVC.VC-V</t>
-  </si>
-  <si>
-    <t>CVC.VC-VC</t>
-  </si>
-  <si>
     <t>8 vowel</t>
   </si>
   <si>
@@ -212,6 +176,24 @@
   </si>
   <si>
     <t>expanded version</t>
+  </si>
+  <si>
+    <t>V-V-CV</t>
+  </si>
+  <si>
+    <t>V-V-VC</t>
+  </si>
+  <si>
+    <t>V-V-CVC</t>
+  </si>
+  <si>
+    <t>V-CV-V</t>
+  </si>
+  <si>
+    <t>V-CV-CV</t>
+  </si>
+  <si>
+    <t>V-CV-VC</t>
   </si>
 </sst>
 </file>
@@ -665,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
@@ -758,40 +740,39 @@
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>54</v>
+      <c r="E5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>4</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="D6" s="2">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2">
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
         <f>B6*C6*D6</f>
         <v>272</v>
       </c>
       <c r="H6" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="J6">
         <f>E6+E7+E8+E9+E10+E11+E12+E13+E14+E15+E16+E17+E18+E19+E20</f>
@@ -799,24 +780,24 @@
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7">
         <v>4</v>
       </c>
-      <c r="C7" s="2">
-        <v>68</v>
-      </c>
-      <c r="D7" s="2">
-        <v>1</v>
-      </c>
-      <c r="E7" s="2">
+      <c r="C7">
+        <v>68</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
         <f>B7*C7*D7</f>
         <v>272</v>
       </c>
       <c r="H7" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="J7">
         <f>E6+E8+E10+E13+E15+E17</f>
@@ -824,539 +805,281 @@
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
+      <c r="A8" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8">
         <v>4</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8">
         <f>17*4*17</f>
         <v>1156</v>
       </c>
-      <c r="D8" s="2">
-        <v>1</v>
-      </c>
-      <c r="E8" s="2">
-        <f t="shared" ref="E8:E36" si="1">B8*C8*D8</f>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <f t="shared" ref="E8:E43" si="1">B8*C8*D8</f>
         <v>4624</v>
       </c>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B9" s="2">
-        <v>68</v>
-      </c>
-      <c r="C9" s="2">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9">
+        <v>68</v>
+      </c>
+      <c r="C9">
         <v>4</v>
       </c>
-      <c r="D9" s="2">
-        <v>1</v>
-      </c>
-      <c r="E9" s="2">
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
         <f t="shared" si="1"/>
         <v>272</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="A10" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="D10" s="2">
-        <v>1</v>
-      </c>
-      <c r="E10" s="2">
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
         <f t="shared" si="1"/>
         <v>4624</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="2">
-        <v>68</v>
-      </c>
-      <c r="C11" s="2">
-        <v>68</v>
-      </c>
-      <c r="D11" s="2">
-        <v>1</v>
-      </c>
-      <c r="E11" s="2">
+      <c r="A11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11">
+        <v>68</v>
+      </c>
+      <c r="C11">
+        <v>68</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+      <c r="E11">
         <f t="shared" si="1"/>
         <v>4624</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
+      <c r="A12" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12">
         <f>17*4*17</f>
         <v>1156</v>
       </c>
-      <c r="D12" s="2">
-        <v>1</v>
-      </c>
-      <c r="E12" s="2">
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
         <f t="shared" si="1"/>
         <v>78608</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
+      <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13">
         <v>4</v>
       </c>
-      <c r="D13" s="2">
-        <v>1</v>
-      </c>
-      <c r="E13" s="2">
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
         <f t="shared" si="1"/>
         <v>272</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="2">
-        <v>68</v>
-      </c>
-      <c r="C14" s="2">
-        <v>68</v>
-      </c>
-      <c r="D14" s="2">
-        <v>1</v>
-      </c>
-      <c r="E14" s="2">
+      <c r="A14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14">
+        <v>68</v>
+      </c>
+      <c r="C14">
+        <v>68</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
         <f t="shared" si="1"/>
         <v>4624</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
+      <c r="A15" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="D15" s="2">
-        <v>1</v>
-      </c>
-      <c r="E15" s="2">
+      <c r="D15">
+        <v>1</v>
+      </c>
+      <c r="E15">
         <f t="shared" si="1"/>
         <v>4624</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" s="2">
-        <v>68</v>
-      </c>
-      <c r="C16" s="2">
+      <c r="A16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16">
+        <v>68</v>
+      </c>
+      <c r="C16">
         <v>1156</v>
       </c>
-      <c r="D16" s="2">
-        <v>1</v>
-      </c>
-      <c r="E16" s="2">
+      <c r="D16">
+        <v>1</v>
+      </c>
+      <c r="E16">
         <f t="shared" si="1"/>
         <v>78608</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="2" t="s">
+      <c r="A17" t="s">
         <v>21</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17">
         <f>17*4*17</f>
         <v>1156</v>
       </c>
-      <c r="C17" s="2">
+      <c r="C17">
         <v>4</v>
       </c>
-      <c r="D17" s="2">
-        <v>1</v>
-      </c>
-      <c r="E17" s="2">
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
         <f t="shared" si="1"/>
         <v>4624</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="B18" s="2">
+      <c r="A18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B18">
         <v>1156</v>
       </c>
-      <c r="C18" s="2">
-        <v>68</v>
-      </c>
-      <c r="D18" s="2">
-        <v>1</v>
-      </c>
-      <c r="E18" s="2">
+      <c r="C18">
+        <v>68</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
         <f t="shared" si="1"/>
         <v>78608</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="2" t="s">
+      <c r="A19" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19">
         <f>17*4*17</f>
         <v>1156</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19">
         <f>17*4</f>
         <v>68</v>
       </c>
-      <c r="D19" s="2">
-        <v>1</v>
-      </c>
-      <c r="E19" s="2">
+      <c r="D19">
+        <v>1</v>
+      </c>
+      <c r="E19">
         <f t="shared" si="1"/>
         <v>78608</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="B20" s="2">
+      <c r="A20" t="s">
+        <v>40</v>
+      </c>
+      <c r="B20">
         <v>1156</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20">
         <v>1156</v>
       </c>
-      <c r="D20" s="2">
-        <v>1</v>
-      </c>
-      <c r="E20" s="2">
+      <c r="D20">
+        <v>1</v>
+      </c>
+      <c r="E20">
         <f t="shared" si="1"/>
         <v>1336336</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>23</v>
-      </c>
-      <c r="B21">
-        <v>4</v>
-      </c>
-      <c r="C21">
-        <v>68</v>
-      </c>
-      <c r="D21">
-        <v>68</v>
-      </c>
-      <c r="E21">
-        <f t="shared" si="1"/>
-        <v>18496</v>
-      </c>
-    </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B22">
-        <v>4</v>
-      </c>
-      <c r="C22">
-        <v>68</v>
-      </c>
-      <c r="D22">
-        <v>1156</v>
-      </c>
-      <c r="E22">
-        <f t="shared" si="1"/>
-        <v>314432</v>
+        <v>46</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>25</v>
-      </c>
-      <c r="B23">
-        <v>4</v>
-      </c>
-      <c r="C23">
-        <v>1156</v>
-      </c>
-      <c r="D23">
-        <v>4</v>
-      </c>
-      <c r="E23">
-        <f t="shared" si="1"/>
-        <v>18496</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
-      </c>
-      <c r="B24">
-        <v>4</v>
-      </c>
-      <c r="C24">
-        <v>1156</v>
-      </c>
-      <c r="D24">
-        <v>68</v>
-      </c>
-      <c r="E24">
-        <f t="shared" si="1"/>
-        <v>314432</v>
+        <v>48</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>27</v>
-      </c>
-      <c r="B25">
-        <v>68</v>
-      </c>
-      <c r="C25">
-        <v>68</v>
-      </c>
-      <c r="D25">
-        <v>68</v>
-      </c>
-      <c r="E25">
-        <f t="shared" si="1"/>
-        <v>314432</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>28</v>
-      </c>
-      <c r="B26">
-        <v>68</v>
-      </c>
-      <c r="C26">
-        <v>68</v>
-      </c>
-      <c r="D26">
-        <v>1156</v>
-      </c>
-      <c r="E26">
-        <f t="shared" si="1"/>
-        <v>5345344</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27">
-        <v>68</v>
-      </c>
-      <c r="C27">
-        <v>1156</v>
-      </c>
-      <c r="D27">
-        <v>4</v>
-      </c>
-      <c r="E27">
-        <f t="shared" si="1"/>
-        <v>314432</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>30</v>
-      </c>
-      <c r="B28">
-        <v>68</v>
-      </c>
-      <c r="C28">
-        <v>1156</v>
-      </c>
-      <c r="D28">
-        <v>68</v>
-      </c>
-      <c r="E28">
-        <f t="shared" si="1"/>
-        <v>5345344</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29">
-        <v>68</v>
-      </c>
-      <c r="C29">
-        <v>4</v>
-      </c>
-      <c r="D29">
-        <v>68</v>
-      </c>
-      <c r="E29">
-        <f t="shared" si="1"/>
-        <v>18496</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30">
-        <v>68</v>
-      </c>
-      <c r="C30">
-        <v>4</v>
-      </c>
-      <c r="D30">
-        <v>1156</v>
-      </c>
-      <c r="E30">
-        <f t="shared" si="1"/>
-        <v>314432</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" t="s">
-        <v>33</v>
-      </c>
-      <c r="B31">
-        <v>68</v>
-      </c>
-      <c r="C31">
-        <v>68</v>
-      </c>
-      <c r="D31">
-        <v>4</v>
-      </c>
-      <c r="E31">
-        <f t="shared" si="1"/>
-        <v>18496</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" t="s">
-        <v>34</v>
-      </c>
-      <c r="B32">
-        <v>68</v>
-      </c>
-      <c r="C32">
-        <v>68</v>
-      </c>
-      <c r="D32">
-        <v>68</v>
-      </c>
-      <c r="E32">
-        <f t="shared" si="1"/>
-        <v>314432</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>35</v>
-      </c>
-      <c r="B33">
-        <v>1156</v>
-      </c>
-      <c r="C33">
-        <v>4</v>
-      </c>
-      <c r="D33">
-        <v>68</v>
-      </c>
-      <c r="E33">
-        <f t="shared" si="1"/>
-        <v>314432</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>36</v>
-      </c>
-      <c r="B34">
-        <v>1156</v>
-      </c>
-      <c r="C34">
-        <v>4</v>
-      </c>
-      <c r="D34">
-        <v>1156</v>
-      </c>
-      <c r="E34">
-        <f t="shared" si="1"/>
-        <v>5345344</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35">
-        <v>1156</v>
-      </c>
-      <c r="C35">
-        <v>68</v>
-      </c>
-      <c r="D35">
-        <v>4</v>
-      </c>
-      <c r="E35">
-        <f t="shared" si="1"/>
-        <v>314432</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36">
-        <v>1156</v>
-      </c>
-      <c r="C36">
-        <v>68</v>
-      </c>
-      <c r="D36">
-        <v>68</v>
-      </c>
-      <c r="E36">
-        <f>B36*C36*D36</f>
-        <v>5345344</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1375,19 +1098,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -1402,10 +1125,10 @@
         <v>13</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>14</v>
@@ -1461,7 +1184,7 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
@@ -1485,7 +1208,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="B6" s="2">
         <v>14</v>
@@ -1628,7 +1351,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B7">
         <v>28</v>
@@ -1646,7 +1369,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B8">
         <v>28</v>

</xml_diff>